<commit_message>
Updating BGDPbES, SYFAFE, and BNVFE
</commit_message>
<xml_diff>
--- a/InputData/elec/BGDPbES/BAU Guaranteed Dispatch Perc by Elec Source.xlsx
+++ b/InputData/elec/BGDPbES/BAU Guaranteed Dispatch Perc by Elec Source.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Dropbox\NEXT Group\90. 개인 폴더\이지우\단기대응\202501 EPS 수요전망\V3\elec\BGDPbES\old\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Desktop\EPS Models\SouthKorea EPS\InputData\elec\BGDPbES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C72E484-782E-4026-86CE-282904789755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D729953D-A9A5-4A0F-97F2-5D4F7785F039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="19308" windowHeight="10500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32625" yWindow="795" windowWidth="33210" windowHeight="14370" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -137,11 +137,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -149,13 +149,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -163,7 +163,7 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -196,7 +196,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -212,9 +212,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -252,9 +252,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -287,26 +287,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -339,26 +322,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -533,49 +499,49 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A11"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:1">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:1">
       <c r="A4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:1">
       <c r="A5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:1">
       <c r="A6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:1">
       <c r="A8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:1">
       <c r="A9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:1">
       <c r="A10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:1">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -593,14 +559,14 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE25"/>
-  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="31.09765625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.09765625" customWidth="1"/>
-    <col min="3" max="3" width="11.296875" customWidth="1"/>
+    <col min="1" max="1" width="31.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.109375" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:31">
       <c r="B1">
         <v>2021</v>
       </c>
@@ -692,7 +658,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:31">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -787,7 +753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:31">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -882,102 +848,102 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:31">
       <c r="A4" t="s">
         <v>25</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="J4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="K4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="L4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="M4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="N4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="O4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="Q4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="R4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="S4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="T4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="U4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="V4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="W4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="X4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="Y4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="Z4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="AA4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="AB4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="AC4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="AD4">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="AE4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.4">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:31">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -1072,7 +1038,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:31">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -1167,7 +1133,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:31">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1262,7 +1228,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:31">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1357,7 +1323,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:31">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1452,7 +1418,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:31">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -1547,7 +1513,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:31">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -1642,7 +1608,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:31">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1737,7 +1703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:31">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1832,7 +1798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:31">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -1927,7 +1893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:31">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -2022,7 +1988,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:31">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -2117,7 +2083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:31">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -2212,7 +2178,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:31">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -2307,7 +2273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:31">
       <c r="A19" t="s">
         <v>26</v>
       </c>
@@ -2402,7 +2368,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="20" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:31">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -2497,7 +2463,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:31">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -2592,7 +2558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:31">
       <c r="A22" t="s">
         <v>29</v>
       </c>
@@ -2687,7 +2653,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:31">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -2782,7 +2748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:31">
       <c r="A24" s="2" t="s">
         <v>31</v>
       </c>
@@ -2877,7 +2843,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:31" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:31">
       <c r="A25" s="2" t="s">
         <v>32</v>
       </c>
@@ -3139,13 +3105,36 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FB8BDF5-EACC-4971-AE10-C3984748F42F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FB8BDF5-EACC-4971-AE10-C3984748F42F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="40f4d404-d193-41dc-bb72-733c1e774208"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{68AEF5D0-07AD-46F0-A983-023B13806554}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{68AEF5D0-07AD-46F0-A983-023B13806554}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F334E6F-B31F-4960-A65A-84336026C096}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F334E6F-B31F-4960-A65A-84336026C096}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updated and calibrated power sector variables. Primarily calibrated wind, solar, nuclear, and natural gas combined cycle.
</commit_message>
<xml_diff>
--- a/InputData/elec/BGDPbES/BAU Guaranteed Dispatch Perc by Elec Source.xlsx
+++ b/InputData/elec/BGDPbES/BAU Guaranteed Dispatch Perc by Elec Source.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Desktop\EPS Models\SouthKorea EPS\InputData\elec\BGDPbES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\South Korea\Models\eps-southkorea\InputData\elec\BGDPbES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D729953D-A9A5-4A0F-97F2-5D4F7785F039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEB2A7AF-84FC-4C5C-A616-339BD181BB00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32625" yWindow="795" windowWidth="33210" windowHeight="14370" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
-    <sheet name="BGDPbES" sheetId="2" r:id="rId2"/>
+    <sheet name="Calibration" sheetId="3" r:id="rId2"/>
+    <sheet name="BGDPbES" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>Notes:</t>
   </si>
@@ -131,13 +132,30 @@
   </si>
   <si>
     <t>hydrogen combined cycle</t>
+  </si>
+  <si>
+    <t>Nuclear</t>
+  </si>
+  <si>
+    <t>Capacity</t>
+  </si>
+  <si>
+    <t>Generation</t>
+  </si>
+  <si>
+    <t>Capacity Factor</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <numFmts count="3">
+    <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="168" formatCode="_(* #,##0.0000_);_(* \(#,##0.0000\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -167,16 +185,36 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -184,18 +222,58 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="11" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="5" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="5" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma [0]" xfId="1" builtinId="6"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -499,7 +577,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A11"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
@@ -554,16 +632,88 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B83E9A6-440E-43CC-A298-E4D6B3B0B543}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1">
+        <v>2021</v>
+      </c>
+      <c r="C1">
+        <v>2022</v>
+      </c>
+      <c r="D1">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="3">
+        <v>23250000</v>
+      </c>
+      <c r="C2" s="4">
+        <v>24650000</v>
+      </c>
+      <c r="D2" s="5">
+        <v>24650000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="6">
+        <v>158015.23000000001</v>
+      </c>
+      <c r="C3" s="7">
+        <v>176054.01199999999</v>
+      </c>
+      <c r="D3" s="8">
+        <v>180494.09599999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="9">
+        <f>(B3/B2)/($D$3/$D$2)</f>
+        <v>0.92817509980987134</v>
+      </c>
+      <c r="C4" s="9">
+        <f t="shared" ref="C4:D4" si="0">(C3/C2)/($D$3/$D$2)</f>
+        <v>0.97540039204384832</v>
+      </c>
+      <c r="D4" s="9">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE25"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="31.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.109375" customWidth="1"/>
-    <col min="3" max="3" width="11.33203125" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.140625" customWidth="1"/>
+    <col min="3" max="3" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:31">
@@ -853,189 +1003,220 @@
         <v>25</v>
       </c>
       <c r="B4">
-        <v>0.6</v>
+        <f>168/142</f>
+        <v>1.1830985915492958</v>
       </c>
       <c r="C4">
-        <v>0.6</v>
+        <v>1.1490445859872611</v>
       </c>
       <c r="D4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="E4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="F4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="G4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="H4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="I4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="J4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="K4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="L4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="M4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="N4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="O4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="P4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="Q4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="R4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="S4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="T4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="U4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="V4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="W4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="X4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="Y4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="Z4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="AA4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="AB4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="AC4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="AD4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="AE4">
-        <v>0.6</v>
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:31">
       <c r="A5" t="s">
         <v>1</v>
       </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="J5">
-        <v>1</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
-      </c>
-      <c r="N5">
-        <v>1</v>
-      </c>
-      <c r="O5">
-        <v>1</v>
-      </c>
-      <c r="P5">
-        <v>1</v>
-      </c>
-      <c r="Q5">
-        <v>1</v>
-      </c>
-      <c r="R5">
-        <v>1</v>
-      </c>
-      <c r="S5">
-        <v>1</v>
-      </c>
-      <c r="T5">
-        <v>1</v>
-      </c>
-      <c r="U5">
-        <v>1</v>
-      </c>
-      <c r="V5">
-        <v>1</v>
-      </c>
-      <c r="W5">
-        <v>1</v>
-      </c>
-      <c r="X5">
-        <v>1</v>
-      </c>
-      <c r="Y5">
-        <v>1</v>
-      </c>
-      <c r="Z5">
-        <v>1</v>
-      </c>
-      <c r="AA5">
-        <v>1</v>
-      </c>
-      <c r="AB5">
-        <v>1</v>
-      </c>
-      <c r="AC5">
-        <v>1</v>
-      </c>
-      <c r="AD5">
-        <v>1</v>
-      </c>
-      <c r="AE5">
-        <v>1</v>
+      <c r="B5" s="10">
+        <f>Calibration!B4</f>
+        <v>0.92817509980987134</v>
+      </c>
+      <c r="C5" s="10">
+        <f>Calibration!C4</f>
+        <v>0.97540039204384832</v>
+      </c>
+      <c r="D5" s="10">
+        <f>Calibration!D4</f>
+        <v>1</v>
+      </c>
+      <c r="E5" s="10">
+        <f>AVERAGE(B5:D5)</f>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="F5" s="10">
+        <f>E5</f>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="G5" s="10">
+        <f t="shared" ref="G5:AE5" si="0">F5</f>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="H5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="I5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="J5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="K5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="L5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="M5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="N5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="O5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="P5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="Q5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="R5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="S5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="T5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="U5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="V5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="W5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="X5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="Y5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="Z5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="AA5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="AB5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="AC5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="AD5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
+      </c>
+      <c r="AE5" s="10">
+        <f t="shared" si="0"/>
+        <v>0.96785849728457318</v>
       </c>
     </row>
     <row r="6" spans="1:31">
@@ -2946,6 +3127,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -3089,7 +3276,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -3098,13 +3285,16 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F334E6F-B31F-4960-A65A-84336026C096}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0FB8BDF5-EACC-4971-AE10-C3984748F42F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3122,19 +3312,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{68AEF5D0-07AD-46F0-A983-023B13806554}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F334E6F-B31F-4960-A65A-84336026C096}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>